<commit_message>
ci: deliver builds locally and to Firebase App Distribution
Channels from docs/SPEC.md (Distribution: local, firebase), rendered by android-engineer render_ci.py: distribute-firebase.yml (stage release to the testers group on push to main), release-artifact.yml (replaces release.yml), tools/ci version and release-notes scripts, tools/export_build.sh, docs/RELEASE.md. versionCode/versionName come from CI (CI-07).

gate (final): build ✓ static-analysis ✓ tests+coverage ✓ rules ✓ ci ✓ dead-code 0 ✓ · test-ratio 0.42

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HANDOVER.xlsx
+++ b/docs/HANDOVER.xlsx
@@ -15,10 +15,10 @@
     <sheet name="Known exceptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Actions'!$A$1:$J$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Secrets &amp; keys'!$A$1:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'External setup'!$A$1:$C$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Verify'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Actions'!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Secrets &amp; keys'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'External setup'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Verify'!$A$1:$B$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Known exceptions'!$A$1:$B$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-15 by android-engineer. Refresh: python3 tools/handover_check.py (keeps the statuses and notes you entered).</t>
+          <t>Generated 2026-10-16 by android-engineer. Refresh: python3 tools/handover_check.py (keeps the statuses and notes you entered).</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>release.yml builds the signed AAB only when these secrets exist (HARD-07).</t>
+          <t>The release workflow (release-artifact.yml or release-play.yml) and the test-build workflows sign only when these secrets exist (HARD-07).</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1196,9 +1196,158 @@
       </c>
       <c r="J10" s="4" t="inlineStr"/>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DIST-1</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Set up Firebase App Distribution for CI</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>distribute-firebase.yml uploads the stage release build to testers with a service account.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>1. Google Cloud console (the Firebase project) → IAM → service account with the role 'Firebase App Distribution Admin' → JSON key → GitHub secret FIREBASE_SERVICE_ACCOUNT_JSON.
+2. Firebase console → App Distribution → Testers &amp; Groups → group 'testers' with the testers' emails.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Push to main (or run the workflow by hand) → testers get an email with the new build</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>DIST-FB-1</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Add the Firebase app id for App Distribution</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>The upload fails with 'Missing app id' until gradle.properties has it (it is not a secret).</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Firebase console → Project settings → Your apps → the Android app com.ilyassavli.helloworld.stage (single environment: com.ilyassavli.helloworld) → App ID (1:…:android:…) → gradle.properties: firebase.stage.appId= (single environment: firebase.appId=).</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>python3 tools/handover_check.py shows this item as Done</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>auto: app id set</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>DIST-LOCAL-1</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Back up the local upload keystore</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>tools/export_build.sh --create-keystore keeps the key in ~/.android-keystores and its passwords in ~/.gradle/gradle.properties — outside the repo. Losing it blocks app updates.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Copy ~/.android-keystores/&lt;project&gt;.jks and the &lt;project&gt;.keystore.* lines from ~/.gradle/gradle.properties into the team's password manager. For CI, base64 it into KEYSTORE_BASE64 with the same passwords.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>The backup restores and tools/export_build.sh signs with it</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
-  <conditionalFormatting sqref="I2:I10">
+  <autoFilter ref="A1:J13"/>
+  <conditionalFormatting sqref="I2:I13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -1210,7 +1359,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I2:I13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"To do,Done,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1224,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1295,7 +1444,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>.github/workflows/release.yml</t>
+          <t>.github/workflows/release-artifact.yml or release-play.yml (+ distribute-*.yml)</t>
         </is>
       </c>
     </row>
@@ -1427,8 +1576,72 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>FIREBASE_SERVICE_ACCOUNT_JSON</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Service account JSON (App Distribution Admin)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>GitHub secret</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Google Cloud console → IAM → service account key</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>.github/workflows/distribute-firebase.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>firebase.stage.appId / firebase.appId</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Firebase App ID of the app that receives test builds (not secret)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>gradle.properties</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>stage (single env: —)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Firebase console → Project settings → Your apps</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>app/build.gradle.kts (firebaseAppDistribution)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1439,7 +1652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1498,8 +1711,25 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Firebase App Distribution</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Tester group 'testers'; service account for CI</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>DIST-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C3"/>
+  <autoFilter ref="A1:C4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1510,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1577,8 +1807,20 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Local export</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>tools/export_build.sh --out &lt;folder&gt; --type apk --install</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>